<commit_message>
Address review comments for CORE-000452
</commit_message>
<xml_diff>
--- a/rules/CORE-000452/negative/01/data/unit-test-coreid-CG0432-negative.xlsx
+++ b/rules/CORE-000452/negative/01/data/unit-test-coreid-CG0432-negative.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JanakiRaman\CORE\Rule_Authoring\core-contributor\rules\CORE-000452\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3862989-3DF6-4144-924F-F6652CAC6533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCA2176C-312A-4C70-9BFB-95AE2A2C4BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="46">
   <si>
     <t>Product</t>
   </si>
@@ -152,6 +152,15 @@
   </si>
   <si>
     <t>Record</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t>CDISC-TEST-006</t>
+  </si>
+  <si>
+    <t>101</t>
   </si>
 </sst>
 </file>
@@ -239,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -260,6 +269,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -614,7 +627,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="11.08984375" customWidth="1"/>
@@ -750,6 +763,63 @@
         <v>41</v>
       </c>
     </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="7">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -757,7 +827,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.7265625" customWidth="1"/>
@@ -912,6 +982,30 @@
       </c>
       <c r="H6" s="6"/>
     </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="8">
+        <v>34</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="9"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>